<commit_message>
Remove misleading 撰写专家 from perf template; clarify Skill naming only
Co-authored-by: misswang122727-gif <misswang122727-gif@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/26年2季度绩效考核模板-王珊珊.xlsx
+++ b/26年2季度绩效考核模板-王珊珊.xlsx
@@ -467,7 +467,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A7"/>
+  <dimension ref="A1:A8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="52" customWidth="1" min="1" max="1"/>
@@ -513,6 +513,13 @@
       <c r="A7" s="2" t="inlineStr">
         <is>
           <t>证据文件路径均相对于本仓库根目录。</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>说明：仓库 skill/*.md 里出现的「需求撰写专家」仅为 Cursor Agent 的技能显示名（YAML name 字段），不是岗位、不是 Q2 正式交付物，绩效考核勿写。</t>
         </is>
       </c>
     </row>
@@ -527,7 +534,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H14"/>
+  <dimension ref="A1:H13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="21" customWidth="1" min="1" max="1"/>
@@ -679,12 +686,12 @@
       </c>
       <c r="B11" s="6" t="inlineStr">
         <is>
-          <t>25%</t>
+          <t>30%</t>
         </is>
       </c>
       <c r="C11" s="6" t="inlineStr">
         <is>
-          <t>PRD v1.0 + SOR v1.2 + 评审报告；七大模块指标可验收表述</t>
+          <t>PRD v1.0 + SOR v1.2；七大模块指标可验收表述；配套 docx 导出</t>
         </is>
       </c>
       <c r="D11" s="6" t="inlineStr"/>
@@ -692,7 +699,7 @@
       <c r="F11" s="6" t="inlineStr"/>
       <c r="G11" s="6" t="inlineStr">
         <is>
-          <t>PRD_人形机器人语音交互系统.md；skill/Voice_AI_Signal_Expert_SOR.md；SOR_Review_Report_墨甲v2.md</t>
+          <t>PRD_人形机器人语音交互系统.md；skill/Voice_AI_Signal_Expert_SOR.md；gen_docs.py → *.docx</t>
         </is>
       </c>
     </row>
@@ -729,7 +736,7 @@
       </c>
       <c r="B13" s="6" t="inlineStr">
         <is>
-          <t>15%</t>
+          <t>20%</t>
         </is>
       </c>
       <c r="C13" s="6" t="inlineStr">
@@ -743,31 +750,6 @@
       <c r="G13" s="6" t="inlineStr">
         <is>
           <t>Vendor_Comparison_墨甲v2.md（12 家画像 + 模块评分）</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="6" t="inlineStr">
-        <is>
-          <t>方法论与导出工具</t>
-        </is>
-      </c>
-      <c r="B14" s="6" t="inlineStr">
-        <is>
-          <t>10%</t>
-        </is>
-      </c>
-      <c r="C14" s="6" t="inlineStr">
-        <is>
-          <t>Skill/SOR 撰写规范；gen_docs 导出 docx</t>
-        </is>
-      </c>
-      <c r="D14" s="6" t="inlineStr"/>
-      <c r="E14" s="6" t="inlineStr"/>
-      <c r="F14" s="6" t="inlineStr"/>
-      <c r="G14" s="6" t="inlineStr">
-        <is>
-          <t>skill/*.md；gen_docs.py；*.docx</t>
         </is>
       </c>
     </row>
@@ -785,13 +767,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F7"/>
+  <dimension ref="A1:F8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
-    <col width="16" customWidth="1" min="2" max="2"/>
-    <col width="17" customWidth="1" min="3" max="3"/>
-    <col width="49" customWidth="1" min="4" max="4"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="19" customWidth="1" min="3" max="3"/>
+    <col width="52" customWidth="1" min="4" max="4"/>
     <col width="37" customWidth="1" min="5" max="5"/>
     <col width="32" customWidth="1" min="6" max="6"/>
   </cols>
@@ -1005,6 +987,36 @@
       <c r="F7" t="inlineStr">
         <is>
           <t>已生成多份 docx 于仓库根目录</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>（非交付）Cursor Skill 配置</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Agent 用 prompt 模板</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>skill/Voice_AI_Signal_Expert_SKILL.md 的 name 含「需求撰写专家」字样</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>skill/*.md</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>仅供 AI 写稿触发，不计入岗位与绩效产出</t>
         </is>
       </c>
     </row>
@@ -3064,96 +3076,96 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2bf078d</t>
+          <t>7633ab5</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Add ASCII filename alias for easier download</t>
+          <t>Revise Q2 perf template: facts from repo only, no fabricated KPIs</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>9a38b9a</t>
+          <t>2bf078d</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Add Q2 2026 performance review workbook with quantitative KPIs</t>
+          <t>Add ASCII filename alias for easier download</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>d48a459</t>
+          <t>9a38b9a</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>墨甲机器人 SOR 评审 v1.2：硬伤修复 + 讯飞/思必驰真实产品线模块级可达性校准 (#3)</t>
+          <t>Add Q2 2026 performance review workbook with quantitative KPIs</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>317ad78</t>
+          <t>d48a459</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Merge pull request #1 from misswang122727-gif/claude/epic-sagan-0t6tX</t>
+          <t>墨甲机器人 SOR 评审 v1.2：硬伤修复 + 讯飞/思必驰真实产品线模块级可达性校准 (#3)</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>1b34aa3</t>
+          <t>317ad78</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Rewrite SOR with full content: real metrics, test methods, acceptance criteria</t>
+          <t>Merge pull request #1 from misswang122727-gif/claude/epic-sagan-0t6tX</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>901e6a9</t>
+          <t>1b34aa3</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Add gen_docs.py script for generating .docx exports</t>
+          <t>Rewrite SOR with full content: real metrics, test methods, acceptance criteria</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>78fd32a</t>
+          <t>901e6a9</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Add .docx exports for PRD, Skill, and SOR (墨甲机器人)</t>
+          <t>Add gen_docs.py script for generating .docx exports</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>c2dd44e</t>
+          <t>78fd32a</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Rewrite Skill + SOR strictly per Claude Skill SOP standard</t>
+          <t>Add .docx exports for PRD, Skill, and SOR (墨甲机器人)</t>
         </is>
       </c>
     </row>

</xml_diff>